<commit_message>
Update login UI and version handling
- Make sync interval API-driven and dynamically configurable.
- Fix EXE version update mechanism without changing existing APIs or tracking logic.
- Remove the unwanted icon from the Company Code field.
- Add a company-related icon to the Company Code field.
- Keep Version visible on the Login page and set its text color to pure white.
- Make the login checkbox text clickable.
- Preserve existing authentication, RBAC, APIs, payloads, and project functionality.
</commit_message>
<xml_diff>
--- a/Monitoring Doc/project_tracker_template.xlsx
+++ b/Monitoring Doc/project_tracker_template.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{598CC071-B23F-42CA-AEF5-AB98736D302B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3345BEB6-7FEE-4110-99D2-A133C4526BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Tracker" sheetId="1" r:id="rId1"/>
-    <sheet name="Legend - Instructions" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>Date</t>
   </si>
@@ -44,27 +43,6 @@
   </si>
   <si>
     <t>Meeting me discuss hua</t>
-  </si>
-  <si>
-    <t>Instructions (kaise use karein):</t>
-  </si>
-  <si>
-    <t>1. 'Date' column me task ki date daalein (jaise 2026-09-02).</t>
-  </si>
-  <si>
-    <t>2. 'Task / Point' column me project ka point/task likhein.</t>
-  </si>
-  <si>
-    <t>3. 'Status' column me dropdown se select karein: Done / Pending / In Progress.</t>
-  </si>
-  <si>
-    <t>4. 'Notes' column optional hai - extra detail ke liye.</t>
-  </si>
-  <si>
-    <t>Row 2 (italic, halke pile color me) ek EXAMPLE row hai - ise dekh kar samjhein format kaisa hona chahiye.</t>
-  </si>
-  <si>
-    <t>Row 3 se aage apna data bharna shuru karein.</t>
   </si>
   <si>
     <t xml:space="preserve">1.fix: make Windows EXE version updates dynamic and reliable. 
@@ -80,14 +58,15 @@
   <si>
     <t xml:space="preserve">1.Make table size wider of application and activity timeline sections can occupy more horizontal space
 2.filters should be there and workday progress should also be shown in percentage level like 51 %
-3.Remove version on login page and company code verify icon fix./ check box fix on login page </t>
+3.Remove version on login page and company code verify icon fix./ check box fix on login page/ remove extra spacing
+4.when log send make it configrable </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -111,17 +90,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -173,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -182,8 +150,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -479,7 +445,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="6"/>
+      <c r="A2" s="4"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2" t="s">
         <v>4</v>
@@ -489,23 +455,23 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="168.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="7">
+      <c r="A3" s="5">
         <v>46267</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>13</v>
+      <c r="B3" s="6" t="s">
+        <v>6</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="3"/>
     </row>
-    <row r="4" spans="1:4" ht="112.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="7">
+    <row r="4" spans="1:4" ht="140.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="5">
         <v>46268</v>
       </c>
-      <c r="B4" s="8" t="s">
-        <v>14</v>
+      <c r="B4" s="6" t="s">
+        <v>7</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -688,59 +654,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A9"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="100" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="5"/>
-    </row>
-    <row r="3" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="5"/>
-    </row>
-    <row r="8" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Improve idle activity tracking and user/device fix
</commit_message>
<xml_diff>
--- a/Monitoring Doc/project_tracker_template.xlsx
+++ b/Monitoring Doc/project_tracker_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3345BEB6-7FEE-4110-99D2-A133C4526BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00AB758C-03C3-4216-AB72-B5F00FAEEB80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="14">
   <si>
     <t>Date</t>
   </si>
@@ -36,30 +36,52 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Notes</t>
-  </si>
-  <si>
     <t>Done</t>
   </si>
   <si>
-    <t>Meeting me discuss hua</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.fix: make Windows EXE version updates dynamic and reliable. 
-2.Add auto-update, pre-update sync, and error reporting
-3.dashboard empty size improve 
-4.Tracking and Start Tracking appear confusing because both relate to tracking.
-It should show a Tracking active rather than both.
- 5.Make company logo dynamic on login 
-6.Add multi-user tracking requirements 
-7.Add automatic application update system
-8. Make a excel make the all points </t>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>bugs</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> discuss </t>
   </si>
   <si>
     <t xml:space="preserve">1.Make table size wider of application and activity timeline sections can occupy more horizontal space
 2.filters should be there and workday progress should also be shown in percentage level like 51 %
 3.Remove version on login page and company code verify icon fix./ check box fix on login page/ remove extra spacing
-4.when log send make it configrable </t>
+ </t>
+  </si>
+  <si>
+    <t>1.fix: make Windows EXE version updates dynamic and reliable
+4.Tracking and Start Tracking appear confusing because both relate to tracking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+1.Add auto-update, pre-update sync, and error reporting.
+2.It should show a Tracking active rather than both.
+ 3.Make company logo dynamic on login .
+4.Add multi-user tracking requirements .
+5.Add automatic application update system.
+6. Make a excel make the all points .</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.when log send make it configrable /screnshot 
+clean from local when upload </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.idle mention on that screen .
+2.document update accordong to 
+iHRMS Tracking . 
+3.Productive applications count .
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. fixing in dashboard user/device popup </t>
   </si>
 </sst>
 </file>
@@ -421,232 +443,323 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="45" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="40" customWidth="1"/>
+    <col min="1" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="45" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="45.54296875" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="4"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="168.5" x14ac:dyDescent="0.35">
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="126.5" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
         <v>46267</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="3"/>
-    </row>
-    <row r="4" spans="1:4" ht="140.5" x14ac:dyDescent="0.35">
+      <c r="B3" s="5"/>
+      <c r="C3" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="154.5" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
         <v>46268</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5"/>
+      <c r="C4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="70.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="5">
+        <v>46269</v>
+      </c>
+      <c r="B5" s="5"/>
+      <c r="C5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="C2:C33" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D33 F2:F33" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Done,Pending,In Progress"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
update doc according to  project
</commit_message>
<xml_diff>
--- a/Monitoring Doc/project_tracker_template.xlsx
+++ b/Monitoring Doc/project_tracker_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00AB758C-03C3-4216-AB72-B5F00FAEEB80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B92BF43-6980-47B7-99F1-84757B3BFEDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -81,7 +81,8 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">1. fixing in dashboard user/device popup </t>
+    <t>1. fixing in dashboard user/device popup 
+2.logout can control with api fix this in dashboard .</t>
   </si>
 </sst>
 </file>
@@ -534,7 +535,7 @@
       <c r="D5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F5" s="3" t="s">

</xml_diff>

<commit_message>
fixing the update not responding
</commit_message>
<xml_diff>
--- a/Monitoring Doc/project_tracker_template.xlsx
+++ b/Monitoring Doc/project_tracker_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B92BF43-6980-47B7-99F1-84757B3BFEDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{223586A7-531D-40E9-911E-2CA463C86499}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
   <si>
     <t>Date</t>
   </si>
@@ -37,9 +37,6 @@
   </si>
   <si>
     <t>Done</t>
-  </si>
-  <si>
-    <t>In Progress</t>
   </si>
   <si>
     <t>bugs</t>
@@ -83,6 +80,18 @@
   <si>
     <t>1. fixing in dashboard user/device popup 
 2.logout can control with api fix this in dashboard .</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. when login start after tracking not start
+2. in hidden icon there is option show to exit .
+</t>
+  </si>
+  <si>
+    <t>1. Not responing show exe file .
+2. there some hang something when start .
+3.Fix the iHRMS Monitor idle/tracking state after Windows Sleep/Resume.
+4. update issue when background update start not make a loop .
+5.idle time issue not update in backend .</t>
   </si>
 </sst>
 </file>
@@ -459,7 +468,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -468,7 +477,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -482,7 +491,7 @@
         <v>3</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>3</v>
@@ -494,13 +503,13 @@
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>3</v>
@@ -512,13 +521,13 @@
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>3</v>
@@ -530,24 +539,30 @@
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="98.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="5">
+        <v>46272</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
       <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
+      <c r="E6" s="6" t="s">
+        <v>14</v>
+      </c>
       <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
idle fixing in backend and database .
</commit_message>
<xml_diff>
--- a/Monitoring Doc/project_tracker_template.xlsx
+++ b/Monitoring Doc/project_tracker_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\ihrms_monitor\Monitoring Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{223586A7-531D-40E9-911E-2CA463C86499}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FC3D9F1-86AC-48E7-9E14-71EA8321ED31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="15">
   <si>
     <t>Date</t>
   </si>
@@ -559,11 +559,15 @@
       <c r="C6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="E6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="3"/>
+      <c r="F6" s="3" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>

</xml_diff>